<commit_message>
Got initial things working
</commit_message>
<xml_diff>
--- a/input_files/input.xlsx
+++ b/input_files/input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yannick\workplace\yannick\hall-scheduler\input_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yanni\workplace\yannick\hall-scheduler\input_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A6D73E-FB13-4604-83C2-CC805FB1172D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11912E25-1F48-417A-8E5A-ACBAC7A19BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hall Space" sheetId="1" r:id="rId1"/>
@@ -39,40 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>J</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
   <si>
     <t>G1</t>
   </si>
@@ -101,12 +68,6 @@
     <t>Friday</t>
   </si>
   <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Unavailable when</t>
   </si>
   <si>
@@ -119,9 +80,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Thursday, Wednesday</t>
-  </si>
-  <si>
     <t>N practices</t>
   </si>
   <si>
@@ -149,19 +107,79 @@
     <t>Slot 7</t>
   </si>
   <si>
-    <t>Slot 8</t>
-  </si>
-  <si>
-    <t>Slot 9</t>
-  </si>
-  <si>
-    <t>Slot 10</t>
-  </si>
-  <si>
     <t>Can make slot 1</t>
   </si>
   <si>
-    <t>No</t>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>Slot</t>
+  </si>
+  <si>
+    <t>G3</t>
+  </si>
+  <si>
+    <t>G4</t>
+  </si>
+  <si>
+    <t>G5</t>
+  </si>
+  <si>
+    <t>G6</t>
+  </si>
+  <si>
+    <t>G7</t>
+  </si>
+  <si>
+    <t>G8</t>
+  </si>
+  <si>
+    <t>G9</t>
+  </si>
+  <si>
+    <t>L4</t>
+  </si>
+  <si>
+    <t>L5</t>
+  </si>
+  <si>
+    <t>L6</t>
+  </si>
+  <si>
+    <t>L7</t>
+  </si>
+  <si>
+    <t>L8</t>
+  </si>
+  <si>
+    <t>L9</t>
+  </si>
+  <si>
+    <t>L10</t>
+  </si>
+  <si>
+    <t>L11</t>
+  </si>
+  <si>
+    <t>L12</t>
+  </si>
+  <si>
+    <t>L13</t>
+  </si>
+  <si>
+    <t>L14</t>
+  </si>
+  <si>
+    <t>L15</t>
+  </si>
+  <si>
+    <t>1.5</t>
   </si>
 </sst>
 </file>
@@ -203,8 +221,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,79 +504,167 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="F1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -568,208 +675,339 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6DE61BE-8B59-42DA-BE76-1985B8C6B693}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.77083333333333337</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.8125</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.89583333333333304</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.85416666666666696</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.95833333333333304</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1">
+        <v>0.875</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.95833333333333337</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84BA844-8809-4554-83D2-EB48A22DC23B}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5">
-        <v>1.5</v>
+      <c r="B11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57A4071-C035-4788-B3D8-8E0CB6A6580C}">
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
         <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Started work on get_primordial_genome function, refactored some code
</commit_message>
<xml_diff>
--- a/input_files/input.xlsx
+++ b/input_files/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yanni\workplace\yannick\hall-scheduler\input_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11912E25-1F48-417A-8E5A-ACBAC7A19BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A14AE9E-47C9-4A6A-9574-2F29285549A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
   <si>
     <t>G1</t>
   </si>
@@ -180,6 +180,12 @@
   </si>
   <si>
     <t>1.5</t>
+  </si>
+  <si>
+    <t>N 2 hours</t>
+  </si>
+  <si>
+    <t>0.5</t>
   </si>
 </sst>
 </file>
@@ -773,207 +779,285 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84BA844-8809-4554-83D2-EB48A22DC23B}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
       <c r="B1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>27</v>
       </c>
       <c r="B4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>30</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>31</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>32</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>25</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>34</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>35</v>
       </c>
       <c r="B15" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>36</v>
       </c>
       <c r="B16" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>37</v>
       </c>
       <c r="B17" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>38</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>39</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>40</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>42</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>43</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>44</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>45</v>
       </c>
       <c r="B25">
         <v>1</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Almost got primordial genome working fully
</commit_message>
<xml_diff>
--- a/input_files/input.xlsx
+++ b/input_files/input.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yanni\workplace\yannick\hall-scheduler\input_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\yannick\workplace\yannick\hall-scheduler\input_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A14AE9E-47C9-4A6A-9574-2F29285549A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB4C1B8-9B8D-4588-8808-30773239A181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hall Space" sheetId="1" r:id="rId1"/>
@@ -182,10 +182,10 @@
     <t>1.5</t>
   </si>
   <si>
-    <t>N 2 hours</t>
-  </si>
-  <si>
     <t>0.5</t>
+  </si>
+  <si>
+    <t>N longer</t>
   </si>
 </sst>
 </file>
@@ -511,9 +511,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -533,7 +533,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -553,7 +553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -593,7 +593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -613,7 +613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -633,7 +633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -653,7 +653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -682,9 +682,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6DE61BE-8B59-42DA-BE76-1985B8C6B693}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -695,7 +695,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -706,7 +706,7 @@
         <v>0.77083333333333337</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -717,7 +717,7 @@
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -728,7 +728,7 @@
         <v>0.89583333333333304</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -739,7 +739,7 @@
         <v>0.95833333333333304</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -750,7 +750,7 @@
         <v>0.85416666666666663</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -761,7 +761,7 @@
         <v>0.95833333333333337</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -780,12 +780,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A84BA844-8809-4554-83D2-EB48A22DC23B}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -793,10 +793,10 @@
         <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -807,7 +807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -818,7 +818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -826,10 +826,10 @@
         <v>46</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -840,7 +840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -851,7 +851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -873,7 +873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -895,7 +895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -906,7 +906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -917,7 +917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -950,7 +950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -961,7 +961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -969,10 +969,10 @@
         <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -983,7 +983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -994,7 +994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>43</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -1069,15 +1069,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57A4071-C035-4788-B3D8-8E0CB6A6580C}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>

</xml_diff>